<commit_message>
Round 1 - Complete
</commit_message>
<xml_diff>
--- a/package-output-map.xlsx
+++ b/package-output-map.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10609"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11027"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/floswald/git/JPEtemplate/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/fra/Desktop/JPE-replications/Reproducibility_Workshop/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{067DD2C7-24FE-2447-A5A8-8F6542C7C06E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{94734606-1ACB-614E-B752-1A98186C8098}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="21900" windowHeight="12060" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="17400" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="7">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="47">
   <si>
     <t>Data Preparation Program</t>
   </si>
@@ -46,6 +46,126 @@
   </si>
   <si>
     <t>In-text numbers</t>
+  </si>
+  <si>
+    <t>Table 1</t>
+  </si>
+  <si>
+    <t>code/quantile_regr/table1.m</t>
+  </si>
+  <si>
+    <t>Table 2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Figure 1Q </t>
+  </si>
+  <si>
+    <t>Figure 1</t>
+  </si>
+  <si>
+    <t>Figure 2</t>
+  </si>
+  <si>
+    <t>Figure 3</t>
+  </si>
+  <si>
+    <t>Figure 4</t>
+  </si>
+  <si>
+    <t>Figure 5</t>
+  </si>
+  <si>
+    <t>Figure 6</t>
+  </si>
+  <si>
+    <t>Figure 7</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Figure 8 </t>
+  </si>
+  <si>
+    <t>down_up_USA.png</t>
+  </si>
+  <si>
+    <t>linear_downside_risk_irf_USA.png</t>
+  </si>
+  <si>
+    <t>comparison_downside_risk_vs_avg_irf_USA.png</t>
+  </si>
+  <si>
+    <t>linear_downside_risk_irf_USA_ECB.png</t>
+  </si>
+  <si>
+    <t>comparison_downside_risk_vs_avg_irf_USA_ECB.png</t>
+  </si>
+  <si>
+    <t>linear_downside_risk_irf_INFO.png</t>
+  </si>
+  <si>
+    <t>comparison_downside_risk_vs_avg_irf_INFO.png</t>
+  </si>
+  <si>
+    <t>comparison_downside_risk_US_FED_vs_ECB.png</t>
+  </si>
+  <si>
+    <t>code/appendix/results_appendix/pred_q_usa.mat</t>
+  </si>
+  <si>
+    <t>yy.mat</t>
+  </si>
+  <si>
+    <t>code/quantile_regr/data_build.m</t>
+  </si>
+  <si>
+    <t>code/quantile_regr/table2.m</t>
+  </si>
+  <si>
+    <t xml:space="preserve">quantile_regr/figure1.m </t>
+  </si>
+  <si>
+    <t>code/figures/figure1.m</t>
+  </si>
+  <si>
+    <t xml:space="preserve">code/figures/figure2.m </t>
+  </si>
+  <si>
+    <t>code/figures/figure2.m</t>
+  </si>
+  <si>
+    <t xml:space="preserve">code/figures/figure5.m </t>
+  </si>
+  <si>
+    <t>code/figures/figure5.m</t>
+  </si>
+  <si>
+    <t>code/figures/figure3.m</t>
+  </si>
+  <si>
+    <t>code/figures/figure4.m</t>
+  </si>
+  <si>
+    <t>code/figures/figure7.m</t>
+  </si>
+  <si>
+    <t xml:space="preserve">code/appendix/quantile_regr_usa.m </t>
+  </si>
+  <si>
+    <t xml:space="preserve">code/appendix/figureA11_usa.m </t>
+  </si>
+  <si>
+    <t xml:space="preserve">code/appendix/figureA1_usa.m </t>
+  </si>
+  <si>
+    <t xml:space="preserve">code/appendix/figureA2_info.m </t>
+  </si>
+  <si>
+    <t xml:space="preserve">code/appendix/figureA3_info.m </t>
+  </si>
+  <si>
+    <t>Yes</t>
+  </si>
+  <si>
+    <t>No</t>
   </si>
 </sst>
 </file>
@@ -434,12 +554,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D18"/>
+  <dimension ref="A1:D26"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="23.5" customWidth="1"/>
-    <col min="2" max="2" width="13.33203125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="41.83203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="39.6640625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="13" customWidth="1"/>
+    <col min="4" max="4" width="11.5" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="12.1640625" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="11.1640625" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="11.5" bestFit="1" customWidth="1"/>
@@ -461,46 +582,318 @@
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A2" s="3"/>
-      <c r="B2" s="3"/>
+      <c r="A2" t="s">
+        <v>29</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="C2" t="s">
+        <v>45</v>
+      </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A3" s="3"/>
-      <c r="B3" s="3"/>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A4" s="3"/>
-      <c r="B4" s="3"/>
+      <c r="A3" t="s">
+        <v>29</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="C3" t="s">
+        <v>45</v>
+      </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A5" s="3"/>
-      <c r="B5" s="3"/>
+      <c r="A5" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A6" t="s">
+        <v>7</v>
+      </c>
+      <c r="B6" t="s">
+        <v>8</v>
+      </c>
+      <c r="C6">
+        <v>40</v>
+      </c>
+      <c r="D6" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A7" t="s">
+        <v>9</v>
+      </c>
+      <c r="B7" t="s">
+        <v>30</v>
+      </c>
+      <c r="C7">
+        <v>467</v>
+      </c>
+      <c r="D7" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A8" t="s">
+        <v>10</v>
+      </c>
+      <c r="B8" t="s">
+        <v>31</v>
+      </c>
+      <c r="C8">
+        <v>57</v>
+      </c>
+      <c r="D8" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A9" t="s">
+        <v>11</v>
+      </c>
+      <c r="B9" t="s">
+        <v>32</v>
+      </c>
+      <c r="C9">
+        <v>90</v>
+      </c>
+      <c r="D9" t="s">
+        <v>45</v>
+      </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A10" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="B10" s="1" t="s">
+      <c r="A10" t="s">
+        <v>12</v>
+      </c>
+      <c r="B10" t="s">
+        <v>33</v>
+      </c>
+      <c r="C10">
+        <v>96</v>
+      </c>
+      <c r="D10" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A11" t="s">
+        <v>13</v>
+      </c>
+      <c r="B11" t="s">
+        <v>34</v>
+      </c>
+      <c r="C11">
+        <v>151</v>
+      </c>
+      <c r="D11" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A12" t="s">
+        <v>14</v>
+      </c>
+      <c r="B12" t="s">
+        <v>35</v>
+      </c>
+      <c r="C12">
+        <v>89</v>
+      </c>
+      <c r="D12" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A13" t="s">
+        <v>15</v>
+      </c>
+      <c r="B13" t="s">
+        <v>36</v>
+      </c>
+      <c r="C13">
+        <v>144</v>
+      </c>
+      <c r="D13" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A14" t="s">
+        <v>16</v>
+      </c>
+      <c r="B14" t="s">
+        <v>37</v>
+      </c>
+      <c r="C14">
+        <v>77</v>
+      </c>
+      <c r="D14" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A15" t="s">
+        <v>17</v>
+      </c>
+      <c r="B15" t="s">
+        <v>38</v>
+      </c>
+      <c r="C15">
+        <v>74</v>
+      </c>
+      <c r="D15" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A16" t="s">
+        <v>18</v>
+      </c>
+      <c r="B16" t="s">
+        <v>39</v>
+      </c>
+      <c r="C16">
+        <v>66</v>
+      </c>
+      <c r="D16" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A17" t="s">
+        <v>19</v>
+      </c>
+      <c r="B17" t="s">
+        <v>40</v>
+      </c>
+      <c r="C17">
+        <v>109</v>
+      </c>
+      <c r="D17" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A18" t="s">
+        <v>20</v>
+      </c>
+      <c r="B18" t="s">
+        <v>41</v>
+      </c>
+      <c r="C18">
+        <v>101</v>
+      </c>
+      <c r="D18" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A19" t="s">
+        <v>21</v>
+      </c>
+      <c r="B19" t="s">
+        <v>41</v>
+      </c>
+      <c r="C19">
+        <v>157</v>
+      </c>
+      <c r="D19" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A20" t="s">
+        <v>22</v>
+      </c>
+      <c r="B20" t="s">
+        <v>42</v>
+      </c>
+      <c r="C20">
+        <v>92</v>
+      </c>
+      <c r="D20" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A21" t="s">
+        <v>23</v>
+      </c>
+      <c r="B21" t="s">
+        <v>42</v>
+      </c>
+      <c r="C21">
+        <v>146</v>
+      </c>
+      <c r="D21" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A22" t="s">
+        <v>24</v>
+      </c>
+      <c r="B22" t="s">
+        <v>43</v>
+      </c>
+      <c r="C22">
+        <v>102</v>
+      </c>
+      <c r="D22" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A23" t="s">
+        <v>25</v>
+      </c>
+      <c r="B23" t="s">
+        <v>43</v>
+      </c>
+      <c r="C23">
+        <v>157</v>
+      </c>
+      <c r="D23" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A24" t="s">
+        <v>26</v>
+      </c>
+      <c r="B24" t="s">
+        <v>44</v>
+      </c>
+      <c r="C24">
+        <v>70</v>
+      </c>
+      <c r="D24" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A26" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B26" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="C10" s="1" t="s">
+      <c r="C26" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="D10" s="2" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A18" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="B18" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="C18" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="D18" s="2" t="s">
+      <c r="D26" s="2" t="s">
         <v>2</v>
       </c>
     </row>

</xml_diff>